<commit_message>
Add Gantt chart export manifest and new Excel prototype file
- Created a new manifest file for the Gantt chart export detailing the source, revision, export date, timeline, page size, and date ranges for each page.
- Added a new Excel file for the JEA Cardboard Prototype, including initial data for Jordan Prunty.
</commit_message>
<xml_diff>
--- a/JEA Cardboard Prototype Tabulated REV1.xlsx
+++ b/JEA Cardboard Prototype Tabulated REV1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jprun\Downloads\JEA Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9114F66-E20E-4E53-B051-3D1FDA39E655}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D08A7FC-4DC4-47FE-95F2-1CAE7B6D8C5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="93">
   <si>
     <t>Node ID</t>
   </si>
@@ -319,6 +319,9 @@
   </si>
   <si>
     <t>N35</t>
+  </si>
+  <si>
+    <t>note</t>
   </si>
 </sst>
 </file>
@@ -1098,7 +1101,7 @@
         <v>40</v>
       </c>
       <c r="B29">
-        <v>40.1</v>
+        <v>41.1</v>
       </c>
       <c r="C29">
         <v>29.03</v>
@@ -1626,7 +1629,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B46BBDD-7595-4ED0-A31A-D2828D973643}">
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
@@ -1655,7 +1658,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -1740,7 +1743,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -1774,7 +1777,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -1825,7 +1828,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -1859,7 +1862,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -1876,7 +1879,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -1905,7 +1908,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1922,12 +1925,12 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -1939,7 +1942,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1956,7 +1959,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1973,7 +1976,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1990,7 +1993,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2007,7 +2010,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2024,7 +2027,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2041,12 +2044,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C25">
         <v>1</v>
@@ -2058,7 +2061,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2066,97 +2069,117 @@
         <v>7</v>
       </c>
       <c r="C26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D26" t="s">
+        <v>40</v>
+      </c>
+      <c r="E26" t="s">
         <v>39</v>
       </c>
-      <c r="E26" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C27">
         <v>1</v>
       </c>
       <c r="D27" t="s">
+        <v>39</v>
+      </c>
+      <c r="E27" t="s">
         <v>90</v>
       </c>
-      <c r="E27" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F27" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C28">
         <v>1</v>
       </c>
       <c r="D28" t="s">
+        <v>90</v>
+      </c>
+      <c r="E28" t="s">
         <v>38</v>
       </c>
-      <c r="E28" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29" t="s">
+        <v>38</v>
+      </c>
+      <c r="E29" t="s">
         <v>28</v>
       </c>
-      <c r="E29" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="C30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D30" t="s">
+        <v>28</v>
+      </c>
+      <c r="E30" t="s">
         <v>91</v>
       </c>
-      <c r="E30" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31">
+        <v>11</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
+      </c>
+      <c r="D31" t="s">
+        <v>91</v>
+      </c>
+      <c r="E31" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32">
         <v>13</v>
       </c>
-      <c r="C31">
-        <v>1</v>
-      </c>
-      <c r="D31" t="s">
+      <c r="C32">
+        <v>1</v>
+      </c>
+      <c r="D32" t="s">
         <v>29</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E32" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Move struct Piece declaration above function prototypes in FLISR_Trainer_REV2.ino to resolve compilation errors in Arduino IDE.
</commit_message>
<xml_diff>
--- a/JEA Cardboard Prototype Tabulated REV1.xlsx
+++ b/JEA Cardboard Prototype Tabulated REV1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jprun\Downloads\JEA Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D08A7FC-4DC4-47FE-95F2-1CAE7B6D8C5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{82C5A16B-77AA-42C1-9C27-C651518672BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Element" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="LED" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="92">
   <si>
     <t>Node ID</t>
   </si>
@@ -319,9 +320,6 @@
   </si>
   <si>
     <t>N35</t>
-  </si>
-  <si>
-    <t>note</t>
   </si>
 </sst>
 </file>
@@ -1629,7 +1627,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B46BBDD-7595-4ED0-A31A-D2828D973643}">
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
@@ -1908,7 +1906,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1925,7 +1923,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1942,7 +1940,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1959,7 +1957,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1976,7 +1974,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1993,7 +1991,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2010,7 +2008,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2027,7 +2025,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2044,7 +2042,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2061,7 +2059,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2078,7 +2076,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2094,11 +2092,8 @@
       <c r="E27" t="s">
         <v>90</v>
       </c>
-      <c r="F27" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2115,7 +2110,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2132,7 +2127,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2149,7 +2144,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2166,7 +2161,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>

</xml_diff>